<commit_message>
Update daily stock valuation report
</commit_message>
<xml_diff>
--- a/data/valuation_history.xlsx
+++ b/data/valuation_history.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P640"/>
+  <dimension ref="A1:P649"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -37059,16 +37059,16 @@
         <v>10.38768</v>
       </c>
       <c r="M632" t="n">
-        <v>0.02624371745869324</v>
+        <v>0.0262437174586932</v>
       </c>
       <c r="N632" t="n">
-        <v>0.02881581244168899</v>
+        <v>0.0288158124416889</v>
       </c>
       <c r="O632" t="n">
-        <v>0.04974999904632568</v>
+        <v>0.0497499990463256</v>
       </c>
       <c r="P632" t="n">
-        <v>-0.02093418660463669</v>
+        <v>-0.0209341866046366</v>
       </c>
     </row>
     <row r="633">
@@ -37117,16 +37117,16 @@
         <v>20.398724</v>
       </c>
       <c r="M633" t="n">
-        <v>0.007614360723073645</v>
+        <v>0.0076143607230736</v>
       </c>
       <c r="N633" t="n">
         <v>0.0300515180284037</v>
       </c>
       <c r="O633" t="n">
-        <v>0.04974999904632568</v>
+        <v>0.0497499990463256</v>
       </c>
       <c r="P633" t="n">
-        <v>-0.01969848101792198</v>
+        <v>-0.0196984810179219</v>
       </c>
     </row>
     <row r="634">
@@ -37175,16 +37175,16 @@
         <v>3.5706854</v>
       </c>
       <c r="M634" t="n">
-        <v>0.048368252979204</v>
+        <v>0.0483682529792039</v>
       </c>
       <c r="N634" t="n">
-        <v>0.04051674585248073</v>
+        <v>0.0405167458524807</v>
       </c>
       <c r="O634" t="n">
-        <v>0.04974999904632568</v>
+        <v>0.0497499990463256</v>
       </c>
       <c r="P634" t="n">
-        <v>-0.009233253193844951</v>
+        <v>-0.0092332531938449</v>
       </c>
     </row>
     <row r="635">
@@ -37233,16 +37233,16 @@
         <v>19.39314</v>
       </c>
       <c r="M635" t="n">
-        <v>0.02163043177988342</v>
+        <v>0.0216304317798834</v>
       </c>
       <c r="N635" t="n">
-        <v>0.05354819193900384</v>
+        <v>0.0535481919390038</v>
       </c>
       <c r="O635" t="n">
-        <v>0.04974999904632568</v>
+        <v>0.0497499990463256</v>
       </c>
       <c r="P635" t="n">
-        <v>0.003798192892678159</v>
+        <v>0.0037981928926781</v>
       </c>
     </row>
     <row r="636">
@@ -37291,16 +37291,16 @@
         <v>9.201266</v>
       </c>
       <c r="M636" t="n">
-        <v>0.05938291846772992</v>
+        <v>0.0593829184677299</v>
       </c>
       <c r="N636" t="n">
         <v>0.0443399314353853</v>
       </c>
       <c r="O636" t="n">
-        <v>0.04974999904632568</v>
+        <v>0.0497499990463256</v>
       </c>
       <c r="P636" t="n">
-        <v>-0.005410067610940379</v>
+        <v>-0.0054100676109403</v>
       </c>
     </row>
     <row r="637">
@@ -37349,16 +37349,16 @@
         <v>7.232781</v>
       </c>
       <c r="M637" t="n">
-        <v>0.04097032544789593</v>
+        <v>0.0409703254478959</v>
       </c>
       <c r="N637" t="n">
-        <v>0.05394759501874914</v>
+        <v>0.0539475950187491</v>
       </c>
       <c r="O637" t="n">
-        <v>0.04974999904632568</v>
+        <v>0.0497499990463256</v>
       </c>
       <c r="P637" t="n">
-        <v>0.004197595972423453</v>
+        <v>0.0041975959724234</v>
       </c>
     </row>
     <row r="638">
@@ -37410,13 +37410,13 @@
         <v>0.0362568851764421</v>
       </c>
       <c r="N638" t="n">
-        <v>0.04756164881060469</v>
+        <v>0.0475616488106046</v>
       </c>
       <c r="O638" t="n">
-        <v>0.04974999904632568</v>
+        <v>0.0497499990463256</v>
       </c>
       <c r="P638" t="n">
-        <v>-0.002188350235720997</v>
+        <v>-0.0021883502357209</v>
       </c>
     </row>
     <row r="639">
@@ -37465,16 +37465,16 @@
         <v>6.662887</v>
       </c>
       <c r="M639" t="n">
-        <v>0.04108527131782946</v>
+        <v>0.0410852713178294</v>
       </c>
       <c r="N639" t="n">
         <v>0.0493657622739018</v>
       </c>
       <c r="O639" t="n">
-        <v>0.04974999904632568</v>
+        <v>0.0497499990463256</v>
       </c>
       <c r="P639" t="n">
-        <v>-0.0003842367724238779</v>
+        <v>-0.0003842367724238</v>
       </c>
     </row>
     <row r="640">
@@ -37523,16 +37523,538 @@
         <v>17.39792</v>
       </c>
       <c r="M640" t="n">
-        <v>0.03619038893215448</v>
+        <v>0.0361903889321544</v>
       </c>
       <c r="N640" t="n">
-        <v>0.07131581840670667</v>
+        <v>0.0713158184067066</v>
       </c>
       <c r="O640" t="n">
-        <v>0.04974999904632568</v>
+        <v>0.0497499990463256</v>
       </c>
       <c r="P640" t="n">
-        <v>0.02156581936038099</v>
+        <v>0.0215658193603809</v>
+      </c>
+    </row>
+    <row r="641">
+      <c r="A641" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B641" t="inlineStr">
+        <is>
+          <t>2026-09-14 17:44:04</t>
+        </is>
+      </c>
+      <c r="C641" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="D641" t="inlineStr">
+        <is>
+          <t>Apple Inc.</t>
+        </is>
+      </c>
+      <c r="E641" t="n">
+        <v>333.08</v>
+      </c>
+      <c r="F641" t="n">
+        <v>4861029515264</v>
+      </c>
+      <c r="G641" t="n">
+        <v>8.710000000000001</v>
+      </c>
+      <c r="H641" t="n">
+        <v>9.582850000000001</v>
+      </c>
+      <c r="I641" t="n">
+        <v>38.2411</v>
+      </c>
+      <c r="J641" t="n">
+        <v>34.757923</v>
+      </c>
+      <c r="K641" t="n">
+        <v>2.61</v>
+      </c>
+      <c r="L641" t="n">
+        <v>10.413004</v>
+      </c>
+      <c r="M641" t="n">
+        <v>0.02614987390416717</v>
+      </c>
+      <c r="N641" t="n">
+        <v>0.028770415515792</v>
+      </c>
+      <c r="O641" t="n">
+        <v>0.04960999965667725</v>
+      </c>
+      <c r="P641" t="n">
+        <v>-0.02083958414088525</v>
+      </c>
+    </row>
+    <row r="642">
+      <c r="A642" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B642" t="inlineStr">
+        <is>
+          <t>2026-09-14 17:44:04</t>
+        </is>
+      </c>
+      <c r="C642" t="inlineStr">
+        <is>
+          <t>AMD</t>
+        </is>
+      </c>
+      <c r="D642" t="inlineStr">
+        <is>
+          <t>Advanced Micro Devices, Inc.</t>
+        </is>
+      </c>
+      <c r="E642" t="n">
+        <v>493.41</v>
+      </c>
+      <c r="F642" t="n">
+        <v>805479514112</v>
+      </c>
+      <c r="G642" t="n">
+        <v>3.92</v>
+      </c>
+      <c r="H642" t="n">
+        <v>15.51049</v>
+      </c>
+      <c r="I642" t="n">
+        <v>125.869896</v>
+      </c>
+      <c r="J642" t="n">
+        <v>31.811373</v>
+      </c>
+      <c r="K642" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="L642" t="n">
+        <v>19.500774</v>
+      </c>
+      <c r="M642" t="n">
+        <v>0.007944711294866338</v>
+      </c>
+      <c r="N642" t="n">
+        <v>0.03143529721732433</v>
+      </c>
+      <c r="O642" t="n">
+        <v>0.04960999965667725</v>
+      </c>
+      <c r="P642" t="n">
+        <v>-0.01817470243935292</v>
+      </c>
+    </row>
+    <row r="643">
+      <c r="A643" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B643" t="inlineStr">
+        <is>
+          <t>2026-09-14 17:44:04</t>
+        </is>
+      </c>
+      <c r="C643" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="D643" t="inlineStr">
+        <is>
+          <t>Amazon.com, Inc.</t>
+        </is>
+      </c>
+      <c r="E643" t="n">
+        <v>253.54</v>
+      </c>
+      <c r="F643" t="n">
+        <v>2734761705472</v>
+      </c>
+      <c r="G643" t="n">
+        <v>12.43</v>
+      </c>
+      <c r="H643" t="n">
+        <v>10.40389</v>
+      </c>
+      <c r="I643" t="n">
+        <v>20.397425</v>
+      </c>
+      <c r="J643" t="n">
+        <v>24.369732</v>
+      </c>
+      <c r="K643" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="L643" t="n">
+        <v>3.5256312</v>
+      </c>
+      <c r="M643" t="n">
+        <v>0.0490257947463911</v>
+      </c>
+      <c r="N643" t="n">
+        <v>0.04103451131971287</v>
+      </c>
+      <c r="O643" t="n">
+        <v>0.04960999965667725</v>
+      </c>
+      <c r="P643" t="n">
+        <v>-0.008575488336964379</v>
+      </c>
+    </row>
+    <row r="644">
+      <c r="A644" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B644" t="inlineStr">
+        <is>
+          <t>2026-09-14 17:44:04</t>
+        </is>
+      </c>
+      <c r="C644" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="D644" t="inlineStr">
+        <is>
+          <t>Broadcom Inc.</t>
+        </is>
+      </c>
+      <c r="E644" t="n">
+        <v>344.72</v>
+      </c>
+      <c r="F644" t="n">
+        <v>1645565706240</v>
+      </c>
+      <c r="G644" t="n">
+        <v>7.83</v>
+      </c>
+      <c r="H644" t="n">
+        <v>19.38391</v>
+      </c>
+      <c r="I644" t="n">
+        <v>44.025543</v>
+      </c>
+      <c r="J644" t="n">
+        <v>17.783823</v>
+      </c>
+      <c r="K644" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="L644" t="n">
+        <v>18.467922</v>
+      </c>
+      <c r="M644" t="n">
+        <v>0.02271408679508006</v>
+      </c>
+      <c r="N644" t="n">
+        <v>0.05623088303550707</v>
+      </c>
+      <c r="O644" t="n">
+        <v>0.04960999965667725</v>
+      </c>
+      <c r="P644" t="n">
+        <v>0.006620883378829823</v>
+      </c>
+    </row>
+    <row r="645">
+      <c r="A645" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B645" t="inlineStr">
+        <is>
+          <t>2026-09-14 17:44:04</t>
+        </is>
+      </c>
+      <c r="C645" t="inlineStr">
+        <is>
+          <t>GOOG</t>
+        </is>
+      </c>
+      <c r="D645" t="inlineStr">
+        <is>
+          <t>Alphabet Inc.</t>
+        </is>
+      </c>
+      <c r="E645" t="n">
+        <v>345.71</v>
+      </c>
+      <c r="F645" t="n">
+        <v>4228010737664</v>
+      </c>
+      <c r="G645" t="n">
+        <v>19.93</v>
+      </c>
+      <c r="H645" t="n">
+        <v>14.87383</v>
+      </c>
+      <c r="I645" t="n">
+        <v>17.34621</v>
+      </c>
+      <c r="J645" t="n">
+        <v>23.242836</v>
+      </c>
+      <c r="K645" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="L645" t="n">
+        <v>9.482694</v>
+      </c>
+      <c r="M645" t="n">
+        <v>0.05764947499349166</v>
+      </c>
+      <c r="N645" t="n">
+        <v>0.04302400856208961</v>
+      </c>
+      <c r="O645" t="n">
+        <v>0.04960999965667725</v>
+      </c>
+      <c r="P645" t="n">
+        <v>-0.006585991094587636</v>
+      </c>
+    </row>
+    <row r="646">
+      <c r="A646" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B646" t="inlineStr">
+        <is>
+          <t>2026-09-14 17:44:04</t>
+        </is>
+      </c>
+      <c r="C646" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="D646" t="inlineStr">
+        <is>
+          <t>Meta Platforms, Inc.</t>
+        </is>
+      </c>
+      <c r="E646" t="n">
+        <v>665.6</v>
+      </c>
+      <c r="F646" t="n">
+        <v>1695620005888</v>
+      </c>
+      <c r="G646" t="n">
+        <v>26.57</v>
+      </c>
+      <c r="H646" t="n">
+        <v>34.95966</v>
+      </c>
+      <c r="I646" t="n">
+        <v>25.050808</v>
+      </c>
+      <c r="J646" t="n">
+        <v>19.039085</v>
+      </c>
+      <c r="K646" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="L646" t="n">
+        <v>7.428882</v>
+      </c>
+      <c r="M646" t="n">
+        <v>0.03991887019230769</v>
+      </c>
+      <c r="N646" t="n">
+        <v>0.05252352764423077</v>
+      </c>
+      <c r="O646" t="n">
+        <v>0.04960999965667725</v>
+      </c>
+      <c r="P646" t="n">
+        <v>0.002913527987553517</v>
+      </c>
+    </row>
+    <row r="647">
+      <c r="A647" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B647" t="inlineStr">
+        <is>
+          <t>2026-09-14 17:44:04</t>
+        </is>
+      </c>
+      <c r="C647" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="D647" t="inlineStr">
+        <is>
+          <t>Microsoft Corporation</t>
+        </is>
+      </c>
+      <c r="E647" t="n">
+        <v>505.41</v>
+      </c>
+      <c r="F647" t="n">
+        <v>3752944992256</v>
+      </c>
+      <c r="G647" t="n">
+        <v>17.94</v>
+      </c>
+      <c r="H647" t="n">
+        <v>23.59268</v>
+      </c>
+      <c r="I647" t="n">
+        <v>28.17224</v>
+      </c>
+      <c r="J647" t="n">
+        <v>21.422323</v>
+      </c>
+      <c r="K647" t="n">
+        <v>1.61</v>
+      </c>
+      <c r="L647" t="n">
+        <v>11.309535</v>
+      </c>
+      <c r="M647" t="n">
+        <v>0.03549593399418294</v>
+      </c>
+      <c r="N647" t="n">
+        <v>0.04668027937713935</v>
+      </c>
+      <c r="O647" t="n">
+        <v>0.04960999965667725</v>
+      </c>
+      <c r="P647" t="n">
+        <v>-0.002929720279537897</v>
+      </c>
+    </row>
+    <row r="648">
+      <c r="A648" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B648" t="inlineStr">
+        <is>
+          <t>2026-09-14 17:44:04</t>
+        </is>
+      </c>
+      <c r="C648" t="inlineStr">
+        <is>
+          <t>NFLX</t>
+        </is>
+      </c>
+      <c r="D648" t="inlineStr">
+        <is>
+          <t>Netflix, Inc.</t>
+        </is>
+      </c>
+      <c r="E648" t="n">
+        <v>80.31999999999999</v>
+      </c>
+      <c r="F648" t="n">
+        <v>334447640576</v>
+      </c>
+      <c r="G648" t="n">
+        <v>3.18</v>
+      </c>
+      <c r="H648" t="n">
+        <v>3.82091</v>
+      </c>
+      <c r="I648" t="n">
+        <v>25.25786</v>
+      </c>
+      <c r="J648" t="n">
+        <v>21.02117</v>
+      </c>
+      <c r="K648" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="L648" t="n">
+        <v>6.9142513</v>
+      </c>
+      <c r="M648" t="n">
+        <v>0.03959163346613546</v>
+      </c>
+      <c r="N648" t="n">
+        <v>0.0475710906374502</v>
+      </c>
+      <c r="O648" t="n">
+        <v>0.04960999965667725</v>
+      </c>
+      <c r="P648" t="n">
+        <v>-0.002038909019227049</v>
+      </c>
+    </row>
+    <row r="649">
+      <c r="A649" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B649" t="inlineStr">
+        <is>
+          <t>2026-09-14 17:44:04</t>
+        </is>
+      </c>
+      <c r="C649" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="D649" t="inlineStr">
+        <is>
+          <t>NVIDIA Corporation</t>
+        </is>
+      </c>
+      <c r="E649" t="n">
+        <v>210.96</v>
+      </c>
+      <c r="F649" t="n">
+        <v>5094050889728</v>
+      </c>
+      <c r="G649" t="n">
+        <v>7.9</v>
+      </c>
+      <c r="H649" t="n">
+        <v>15.61489</v>
+      </c>
+      <c r="I649" t="n">
+        <v>26.703798</v>
+      </c>
+      <c r="J649" t="n">
+        <v>13.510182</v>
+      </c>
+      <c r="K649" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="L649" t="n">
+        <v>16.813713</v>
+      </c>
+      <c r="M649" t="n">
+        <v>0.03744785741372772</v>
+      </c>
+      <c r="N649" t="n">
+        <v>0.0740182499051953</v>
+      </c>
+      <c r="O649" t="n">
+        <v>0.04960999965667725</v>
+      </c>
+      <c r="P649" t="n">
+        <v>0.02440825024851805</v>
       </c>
     </row>
   </sheetData>
@@ -37634,12 +38156,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-11 17:24:28</t>
+          <t>2026-09-14 17:44:04</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -37653,51 +38175,51 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>335.45</v>
+        <v>345.71</v>
       </c>
       <c r="F2" t="n">
-        <v>4102531842048</v>
+        <v>4228010737664</v>
       </c>
       <c r="G2" t="n">
-        <v>19.92</v>
+        <v>19.93</v>
       </c>
       <c r="H2" t="n">
         <v>14.87383</v>
       </c>
       <c r="I2" t="n">
-        <v>16.83986</v>
+        <v>17.34621</v>
       </c>
       <c r="J2" t="n">
-        <v>22.553036</v>
+        <v>23.242836</v>
       </c>
       <c r="K2" t="n">
-        <v>1.21</v>
+        <v>1.2</v>
       </c>
       <c r="L2" t="n">
-        <v>9.201266</v>
+        <v>9.482694</v>
       </c>
       <c r="M2" t="n">
-        <v>0.05938291846772992</v>
+        <v>0.05764947499349166</v>
       </c>
       <c r="N2" t="n">
-        <v>0.0443399314353853</v>
+        <v>0.04302400856208961</v>
       </c>
       <c r="O2" t="n">
-        <v>0.04974999904632568</v>
+        <v>0.04960999965667725</v>
       </c>
       <c r="P2" t="n">
-        <v>-0.005410067610940379</v>
+        <v>-0.006585991094587636</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-09-11 17:24:28</t>
+          <t>2026-09-14 17:44:04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -37711,51 +38233,51 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>495.63</v>
+        <v>505.41</v>
       </c>
       <c r="F3" t="n">
-        <v>3680323239936</v>
+        <v>3752944992256</v>
       </c>
       <c r="G3" t="n">
-        <v>17.97</v>
+        <v>17.94</v>
       </c>
       <c r="H3" t="n">
-        <v>23.57298</v>
+        <v>23.59268</v>
       </c>
       <c r="I3" t="n">
-        <v>27.580969</v>
+        <v>28.17224</v>
       </c>
       <c r="J3" t="n">
-        <v>21.025343</v>
+        <v>21.422323</v>
       </c>
       <c r="K3" t="n">
-        <v>1.6</v>
+        <v>1.61</v>
       </c>
       <c r="L3" t="n">
-        <v>11.090689</v>
+        <v>11.309535</v>
       </c>
       <c r="M3" t="n">
-        <v>0.0362568851764421</v>
+        <v>0.03549593399418294</v>
       </c>
       <c r="N3" t="n">
-        <v>0.04756164881060469</v>
+        <v>0.04668027937713935</v>
       </c>
       <c r="O3" t="n">
-        <v>0.04974999904632568</v>
+        <v>0.04960999965667725</v>
       </c>
       <c r="P3" t="n">
-        <v>-0.002188350235720997</v>
+        <v>-0.002929720279537897</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-11 17:24:28</t>
+          <t>2026-09-14 17:44:04</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -37769,51 +38291,51 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>648.03</v>
+        <v>665.6</v>
       </c>
       <c r="F4" t="n">
-        <v>1650860490752</v>
+        <v>1695620005888</v>
       </c>
       <c r="G4" t="n">
-        <v>26.55</v>
+        <v>26.57</v>
       </c>
       <c r="H4" t="n">
         <v>34.95966</v>
       </c>
       <c r="I4" t="n">
-        <v>24.407911</v>
+        <v>25.050808</v>
       </c>
       <c r="J4" t="n">
-        <v>18.536509</v>
+        <v>19.039085</v>
       </c>
       <c r="K4" t="n">
         <v>0.86</v>
       </c>
       <c r="L4" t="n">
-        <v>7.232781</v>
+        <v>7.428882</v>
       </c>
       <c r="M4" t="n">
-        <v>0.04097032544789593</v>
+        <v>0.03991887019230769</v>
       </c>
       <c r="N4" t="n">
-        <v>0.05394759501874914</v>
+        <v>0.05252352764423077</v>
       </c>
       <c r="O4" t="n">
-        <v>0.04974999904632568</v>
+        <v>0.04960999965667725</v>
       </c>
       <c r="P4" t="n">
-        <v>0.004197595972423453</v>
+        <v>0.002913527987553517</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-09-11 17:24:28</t>
+          <t>2026-09-14 17:44:04</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -37827,51 +38349,51 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>256.78</v>
+        <v>253.54</v>
       </c>
       <c r="F5" t="n">
-        <v>2769709432832</v>
+        <v>2734761705472</v>
       </c>
       <c r="G5" t="n">
-        <v>12.42</v>
+        <v>12.43</v>
       </c>
       <c r="H5" t="n">
         <v>10.40389</v>
       </c>
       <c r="I5" t="n">
-        <v>20.674719</v>
+        <v>20.397425</v>
       </c>
       <c r="J5" t="n">
-        <v>24.681154</v>
+        <v>24.369732</v>
       </c>
       <c r="K5" t="n">
-        <v>1.48</v>
+        <v>1.5</v>
       </c>
       <c r="L5" t="n">
-        <v>3.5706854</v>
+        <v>3.5256312</v>
       </c>
       <c r="M5" t="n">
-        <v>0.048368252979204</v>
+        <v>0.0490257947463911</v>
       </c>
       <c r="N5" t="n">
-        <v>0.04051674585248073</v>
+        <v>0.04103451131971287</v>
       </c>
       <c r="O5" t="n">
-        <v>0.04974999904632568</v>
+        <v>0.04960999965667725</v>
       </c>
       <c r="P5" t="n">
-        <v>-0.009233253193844951</v>
+        <v>-0.008575488336964379</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-09-11 17:24:28</t>
+          <t>2026-09-14 17:44:04</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -37885,51 +38407,51 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>332.27</v>
+        <v>333.08</v>
       </c>
       <c r="F6" t="n">
-        <v>4849207869440</v>
+        <v>4861029515264</v>
       </c>
       <c r="G6" t="n">
-        <v>8.720000000000001</v>
+        <v>8.710000000000001</v>
       </c>
       <c r="H6" t="n">
-        <v>9.574630000000001</v>
+        <v>9.582850000000001</v>
       </c>
       <c r="I6" t="n">
-        <v>38.104355</v>
+        <v>38.2411</v>
       </c>
       <c r="J6" t="n">
-        <v>34.703167</v>
+        <v>34.757923</v>
       </c>
       <c r="K6" t="n">
-        <v>2.48</v>
+        <v>2.61</v>
       </c>
       <c r="L6" t="n">
-        <v>10.38768</v>
+        <v>10.413004</v>
       </c>
       <c r="M6" t="n">
-        <v>0.02624371745869324</v>
+        <v>0.02614987390416717</v>
       </c>
       <c r="N6" t="n">
-        <v>0.02881581244168899</v>
+        <v>0.028770415515792</v>
       </c>
       <c r="O6" t="n">
-        <v>0.04974999904632568</v>
+        <v>0.04960999965667725</v>
       </c>
       <c r="P6" t="n">
-        <v>-0.02093418660463669</v>
+        <v>-0.02083958414088525</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-09-11 17:24:28</t>
+          <t>2026-09-14 17:44:04</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -37943,51 +38465,51 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>218.29</v>
+        <v>210.96</v>
       </c>
       <c r="F7" t="n">
-        <v>5271048421376</v>
+        <v>5094050889728</v>
       </c>
       <c r="G7" t="n">
         <v>7.9</v>
       </c>
       <c r="H7" t="n">
-        <v>15.56753</v>
+        <v>15.61489</v>
       </c>
       <c r="I7" t="n">
-        <v>27.631645</v>
+        <v>26.703798</v>
       </c>
       <c r="J7" t="n">
-        <v>14.022135</v>
+        <v>13.510182</v>
       </c>
       <c r="K7" t="n">
-        <v>0.59</v>
+        <v>0.46</v>
       </c>
       <c r="L7" t="n">
-        <v>17.39792</v>
+        <v>16.813713</v>
       </c>
       <c r="M7" t="n">
-        <v>0.03619038893215448</v>
+        <v>0.03744785741372772</v>
       </c>
       <c r="N7" t="n">
-        <v>0.07131581840670667</v>
+        <v>0.0740182499051953</v>
       </c>
       <c r="O7" t="n">
-        <v>0.04974999904632568</v>
+        <v>0.04960999965667725</v>
       </c>
       <c r="P7" t="n">
-        <v>0.02156581936038099</v>
+        <v>0.02440825024851805</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-09-11 17:24:28</t>
+          <t>2026-09-14 17:44:04</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -38001,51 +38523,51 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>516.13</v>
+        <v>493.41</v>
       </c>
       <c r="F8" t="n">
-        <v>842569351168</v>
+        <v>805479514112</v>
       </c>
       <c r="G8" t="n">
-        <v>3.93</v>
+        <v>3.92</v>
       </c>
       <c r="H8" t="n">
         <v>15.51049</v>
       </c>
       <c r="I8" t="n">
-        <v>131.3308</v>
+        <v>125.869896</v>
       </c>
       <c r="J8" t="n">
-        <v>33.276188</v>
+        <v>31.811373</v>
       </c>
       <c r="K8" t="n">
-        <v>0.49</v>
+        <v>0.53</v>
       </c>
       <c r="L8" t="n">
-        <v>20.398724</v>
+        <v>19.500774</v>
       </c>
       <c r="M8" t="n">
-        <v>0.007614360723073645</v>
+        <v>0.007944711294866338</v>
       </c>
       <c r="N8" t="n">
-        <v>0.0300515180284037</v>
+        <v>0.03143529721732433</v>
       </c>
       <c r="O8" t="n">
-        <v>0.04974999904632568</v>
+        <v>0.04960999965667725</v>
       </c>
       <c r="P8" t="n">
-        <v>-0.01969848101792198</v>
+        <v>-0.01817470243935292</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-09-11 17:24:28</t>
+          <t>2026-09-14 17:44:04</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -38059,10 +38581,10 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>361.99</v>
+        <v>344.72</v>
       </c>
       <c r="F9" t="n">
-        <v>1728006324224</v>
+        <v>1645565706240</v>
       </c>
       <c r="G9" t="n">
         <v>7.83</v>
@@ -38071,39 +38593,39 @@
         <v>19.38391</v>
       </c>
       <c r="I9" t="n">
-        <v>46.231163</v>
+        <v>44.025543</v>
       </c>
       <c r="J9" t="n">
-        <v>18.674767</v>
+        <v>17.783823</v>
       </c>
       <c r="K9" t="n">
         <v>0.36</v>
       </c>
       <c r="L9" t="n">
-        <v>19.39314</v>
+        <v>18.467922</v>
       </c>
       <c r="M9" t="n">
-        <v>0.02163043177988342</v>
+        <v>0.02271408679508006</v>
       </c>
       <c r="N9" t="n">
-        <v>0.05354819193900384</v>
+        <v>0.05623088303550707</v>
       </c>
       <c r="O9" t="n">
-        <v>0.04974999904632568</v>
+        <v>0.04960999965667725</v>
       </c>
       <c r="P9" t="n">
-        <v>0.003798192892678159</v>
+        <v>0.006620883378829823</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-09-11 17:24:28</t>
+          <t>2026-09-14 17:44:04</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -38117,10 +38639,10 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>77.40000000000001</v>
+        <v>80.31999999999999</v>
       </c>
       <c r="F10" t="n">
-        <v>322288943104</v>
+        <v>334447640576</v>
       </c>
       <c r="G10" t="n">
         <v>3.18</v>
@@ -38129,28 +38651,28 @@
         <v>3.82091</v>
       </c>
       <c r="I10" t="n">
-        <v>24.339622</v>
+        <v>25.25786</v>
       </c>
       <c r="J10" t="n">
-        <v>20.256954</v>
+        <v>21.02117</v>
       </c>
       <c r="K10" t="n">
-        <v>1.41</v>
+        <v>1.43</v>
       </c>
       <c r="L10" t="n">
-        <v>6.662887</v>
+        <v>6.9142513</v>
       </c>
       <c r="M10" t="n">
-        <v>0.04108527131782946</v>
+        <v>0.03959163346613546</v>
       </c>
       <c r="N10" t="n">
-        <v>0.0493657622739018</v>
+        <v>0.0475710906374502</v>
       </c>
       <c r="O10" t="n">
-        <v>0.04974999904632568</v>
+        <v>0.04960999965667725</v>
       </c>
       <c r="P10" t="n">
-        <v>-0.0003842367724238779</v>
+        <v>-0.002038909019227049</v>
       </c>
     </row>
   </sheetData>

</xml_diff>